<commit_message>
fix: align Gemini debug setting in environment sample fix: correct email instruction in agent rules chore: harden backup creation and validation chore: exclude secrets and virtual environments from backups chore: ignore testing scenarios in workspace setup chore: align formatting in setup and orchestrator scripts
Update .env.sample, brahe-ai-general-rules.xlsx, brahe-ai.py, and 2 more files
</commit_message>
<xml_diff>
--- a/assets/rules/brahe-ai-general-rules.xlsx
+++ b/assets/rules/brahe-ai-general-rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\brahe-ai\brahe-ai-0.1\rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17fefaed0f170910/Personal Managed/Brahe-ai/brahe-ai-workspace/assets/rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57E224D-856D-4CEF-AD19-82A6F5D666DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{A57E224D-856D-4CEF-AD19-82A6F5D666DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D260B561-8C32-4B3A-B6CA-BD26B1A61DDD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agent" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>Value</t>
   </si>
@@ -117,25 +117,13 @@
     <t>xpandas</t>
   </si>
   <si>
-    <t>En base a la columna "departamento" del dataframe , determina cuántos departamentos distintos hay. Para cada departamento detectado, añade una nueva hoja al dataframe con el nombre del departamento y, a esa hoja, añade todas las files que pertenezcan al departamento. Recuerda que la primera fila de las hojas creadas debe contener los nombres de las columnas</t>
-  </si>
-  <si>
-    <t>Ordena el dataframe por las siguientes columnas: primero "departamento" (ascendiente) y luego "inv actual en pzas" (descendiente)</t>
-  </si>
-  <si>
-    <t>Remueve todas las filas del dataframe en donde el "departamento" sea "57-ORGANIZACIÓN"</t>
-  </si>
-  <si>
     <t>read_and_insight</t>
   </si>
   <si>
     <t>Genera un script python que será invocado vía exec y que por medio de llamadas a pandas interactue con dataframe pandas cargado en la variable 'df' con fin de cumplir lo siguiente: "{value}"</t>
   </si>
   <si>
-    <t>Lee el dataframe y genera un email indicando cuántos registros hay por cada departamento. El email debe ser enviado a marc.bonet.bretto@gmail.comy la lista de departamentos debe ser ordenada alfabéticamente. Para el envío del email tendras en el contexto de exec un servicio llamado "google_service". Este servicio tiene un método de envío de emails con la siguiente firma: def send_email(self, to_emails: str, subject: str, body: str, cc_emails: str = None, attachment_path: str = None). Úsalo</t>
-  </si>
-  <si>
-    <t>Eres un motor de generación de código experto en Python y Pandas. Tu única tarea generar un script de python que contenga las instrucciones necesarias para actualizar o leer un dataframe de pandas referenciado por la variable 'df'. Debes generar el script completo y las llamadas a pandas.  El código que generes será ejecutado dentro de otro script python por medio de la instrucción exec; el 'df' mencionado será pasado a exec dentro del contexto local (3er argumento).
+    <t>Eres un motor de generación de código experto en Python y Pandas. Tu única tarea es generar un script de python que contenga las instrucciones necesarias para actualizar o leer un dataframe de pandas referenciado por la variable 'df'. Debes generar el script completo y las llamadas a pandas.  El código que generes será ejecutado dentro de otro script python por medio de la instrucción exec; el 'df' mencionado será pasado a exec dentro del contexto local (3er argumento).
 REGLAS ESTRICTAS:
 1. Asume que el DataFrame ya existe y se llama 'df'.
 2. No cargues el archivo tú mismo ni uses pd.read_excel.
@@ -143,6 +131,21 @@
 4. Devuelve EXCLUSIVAMENTE código python limpio y listo para compilar y luego ejecutar vía exec. No incluyas explicaciones, saludos, ni nada adicional. 
 5. FORMATO: Devuelve el script formateado con saltos de línea reales (físicos). NO devuelvas el código en una sola línea usando caracteres '\n'.
 6. RESTRICCIÓN: No envuelvas el código en estructuras JSON ni formatos de texto plano simulados.</t>
+  </si>
+  <si>
+    <t>ss</t>
+  </si>
+  <si>
+    <t>Lee el dataframe y genera un email indicando cuántos registros hay por cada departamento. El email debe ser enviado a marc.bonet.bretto@gmail.com y la lista de departamentos debe ser ordenada alfabéticamente. Para el envío del email tendras en el contexto de exec un servicio llamado "google_service". Este servicio tiene un método de envío de emails con la siguiente firma: def send_email(self, to_emails: str, subject: str, body: str, cc_emails: str = None, attachment_path: str = None). Úsalo.</t>
+  </si>
+  <si>
+    <t>En base a la columna "departamento" del dataframe , determina cuántos departamentos distintos hay. Para cada departamento detectado, añade una nueva hoja al dataframe con el nombre del departamento y, a esa hoja, añade todas las files que pertenezcan al departamento. Recuerda que la primera fila de las hojas creadas debe contener los nombres de las columnas.</t>
+  </si>
+  <si>
+    <t>Remueve todas las filas del dataframe en donde el "departamento" sea "57-ORGANIZACIÓN".</t>
+  </si>
+  <si>
+    <t>Ordena el dataframe por las siguientes columnas: primero "departamento" (ascendiente) y luego "inv actual en pzas" (descendiente).</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -205,6 +208,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -221,6 +230,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -491,18 +504,18 @@
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="197.42578125" style="6" customWidth="1"/>
     <col min="4" max="4" width="108.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1"/>
@@ -514,7 +527,7 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -525,8 +538,8 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>16</v>
+      <c r="C3" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -536,30 +549,30 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C5" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -600,13 +613,13 @@
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E2" s="3"/>
     </row>

</xml_diff>

<commit_message>
fix: restore Agent rules realm header
Update brahe-ai-general-rules.xlsx
</commit_message>
<xml_diff>
--- a/assets/rules/brahe-ai-general-rules.xlsx
+++ b/assets/rules/brahe-ai-general-rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17fefaed0f170910/Personal Managed/Brahe-ai/brahe-ai-workspace/assets/rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{A57E224D-856D-4CEF-AD19-82A6F5D666DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D260B561-8C32-4B3A-B6CA-BD26B1A61DDD}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{A57E224D-856D-4CEF-AD19-82A6F5D666DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AA0EA11-D48E-4175-86A4-6A536D57DEFB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Value</t>
   </si>
@@ -131,9 +131,6 @@
 4. Devuelve EXCLUSIVAMENTE código python limpio y listo para compilar y luego ejecutar vía exec. No incluyas explicaciones, saludos, ni nada adicional. 
 5. FORMATO: Devuelve el script formateado con saltos de línea reales (físicos). NO devuelvas el código en una sola línea usando caracteres '\n'.
 6. RESTRICCIÓN: No envuelvas el código en estructuras JSON ni formatos de texto plano simulados.</t>
-  </si>
-  <si>
-    <t>ss</t>
   </si>
   <si>
     <t>Lee el dataframe y genera un email indicando cuántos registros hay por cada departamento. El email debe ser enviado a marc.bonet.bretto@gmail.com y la lista de departamentos debe ser ordenada alfabéticamente. Para el envío del email tendras en el contexto de exec un servicio llamado "google_service". Este servicio tiene un método de envío de emails con la siguiente firma: def send_email(self, to_emails: str, subject: str, body: str, cc_emails: str = None, attachment_path: str = None). Úsalo.</t>
@@ -510,7 +507,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -539,7 +536,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -550,7 +547,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -561,7 +558,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -572,7 +569,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>